<commit_message>
Add a bit more to thesis
</commit_message>
<xml_diff>
--- a/Research/TheProjectKaggle/leaderboardanalysis/Topgold/Whatworkeddidntwork.xlsx
+++ b/Research/TheProjectKaggle/leaderboardanalysis/Topgold/Whatworkeddidntwork.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shwes\Projects\Thesis\Research\TheProjectKaggle\leaderboardanalysis\Topgold\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0864C15-91F0-405E-A10B-5C9209D5EC8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B30AD456-A121-437A-8BF4-394B0EB34984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Place Focused" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="171">
   <si>
     <t>Placement</t>
   </si>
@@ -547,6 +547,9 @@
   </si>
   <si>
     <t>more complicated Training Technique did not help as much as better data and preprocessing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ensembled a ByT5-Large and a ByT5-XL model, using a fine-tuned Qwen3-8B pairwise Reward Model to select the better translation per sentence, </t>
   </si>
 </sst>
 </file>
@@ -582,7 +585,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -601,6 +604,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -614,11 +623,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -947,9 +957,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+    <row r="4" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="4" t="s">
         <v>5</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
Add more to thesis, have chappy rephrase that bit
</commit_message>
<xml_diff>
--- a/Research/TheProjectKaggle/leaderboardanalysis/Topgold/Whatworkeddidntwork.xlsx
+++ b/Research/TheProjectKaggle/leaderboardanalysis/Topgold/Whatworkeddidntwork.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shwes\Projects\Thesis\Research\TheProjectKaggle\leaderboardanalysis\Topgold\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B30AD456-A121-437A-8BF4-394B0EB34984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24BB4C1C-AB94-4FB2-BA55-C3CEDB965EE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Place Focused" sheetId="1" r:id="rId1"/>
@@ -1153,154 +1153,166 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B3">
-        <v>9</v>
+        <v>91</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B4">
-        <v>9</v>
+        <v>88</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E4" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B5">
-        <v>11</v>
+        <v>90</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
       </c>
       <c r="D5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E5" t="s">
-        <v>148</v>
+        <v>156</v>
+      </c>
+      <c r="F5" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="C6">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E6" t="s">
-        <v>148</v>
+        <v>157</v>
+      </c>
+      <c r="F6" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>56</v>
-      </c>
-      <c r="B7">
-        <v>5</v>
+        <v>93</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
       </c>
       <c r="D7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E7" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="C8">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E8" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="C9">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E9" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10">
-        <v>1</v>
+        <v>96</v>
+      </c>
+      <c r="C10">
+        <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E10" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>148</v>
+        <v>168</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>144</v>
+        <v>38</v>
       </c>
       <c r="C12">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D12" t="s">
         <v>147</v>
       </c>
       <c r="E12" t="s">
-        <v>148</v>
+        <v>168</v>
+      </c>
+      <c r="F12" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>40</v>
-      </c>
-      <c r="B13">
-        <v>1</v>
+        <v>108</v>
+      </c>
+      <c r="C13">
+        <v>6</v>
       </c>
       <c r="D13" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E13" t="s">
         <v>148</v>
@@ -1308,290 +1320,279 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>59</v>
-      </c>
-      <c r="B14">
+        <v>107</v>
+      </c>
+      <c r="C14">
         <v>6</v>
       </c>
       <c r="D14" t="s">
         <v>148</v>
       </c>
       <c r="E14" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A15" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B15">
-        <v>5</v>
-      </c>
-      <c r="D15" t="s">
-        <v>148</v>
-      </c>
-      <c r="E15" t="s">
-        <v>155</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="A15" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3">
+        <v>6</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A16" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3">
+        <v>6</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
-        <v>65</v>
-      </c>
-      <c r="B16">
+    <row r="17" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="3">
         <v>8</v>
       </c>
-      <c r="D16" t="s">
-        <v>152</v>
-      </c>
-      <c r="E16" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
-        <v>126</v>
-      </c>
-      <c r="C17">
-        <v>12</v>
-      </c>
-      <c r="D17" t="s">
-        <v>152</v>
-      </c>
-      <c r="E17" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
-        <v>73</v>
-      </c>
-      <c r="B18">
-        <v>15</v>
-      </c>
-      <c r="D18" t="s">
-        <v>152</v>
-      </c>
-      <c r="E18" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
-        <v>50</v>
-      </c>
-      <c r="B19">
-        <v>2</v>
-      </c>
-      <c r="D19" t="s">
-        <v>152</v>
-      </c>
-      <c r="E19" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="C17" s="3">
+        <v>6</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A18" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3">
+        <v>6</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A19" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3">
+        <v>6</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="C20">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D20" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E20" t="s">
-        <v>155</v>
-      </c>
-      <c r="F20" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>137</v>
+        <v>112</v>
       </c>
       <c r="C21">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D21" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E21" t="s">
-        <v>155</v>
-      </c>
-      <c r="F21" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>139</v>
+        <v>114</v>
       </c>
       <c r="C22">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D22" t="s">
         <v>149</v>
       </c>
       <c r="E22" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F22" t="s">
-        <v>158</v>
-      </c>
-      <c r="G22" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>51</v>
-      </c>
-      <c r="B23">
-        <v>2</v>
+        <v>116</v>
+      </c>
+      <c r="C23">
+        <v>9</v>
       </c>
       <c r="D23" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E23" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F23" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="C24">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D24" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E24" t="s">
-        <v>155</v>
-      </c>
-      <c r="F24" t="s">
-        <v>158</v>
-      </c>
-      <c r="G24" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B25">
-        <v>8</v>
+        <v>165</v>
+      </c>
+      <c r="C25">
+        <v>9</v>
       </c>
       <c r="D25" t="s">
         <v>147</v>
       </c>
       <c r="E25" t="s">
-        <v>155</v>
-      </c>
-      <c r="F25" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C26">
         <v>9</v>
       </c>
       <c r="D26" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="E26" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>69</v>
-      </c>
-      <c r="B27">
-        <v>8</v>
+        <v>122</v>
       </c>
       <c r="C27">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E27" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>96</v>
+        <v>41</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
       </c>
       <c r="C28">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D28" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E28" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A29" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A29" t="s">
+        <v>121</v>
+      </c>
+      <c r="C29">
+        <v>11</v>
+      </c>
+      <c r="D29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E29" t="s">
+        <v>155</v>
+      </c>
+      <c r="F29" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>119</v>
-      </c>
-      <c r="C30" t="s">
-        <v>146</v>
+        <v>120</v>
+      </c>
+      <c r="C30">
+        <v>11</v>
       </c>
       <c r="D30" t="s">
         <v>147</v>
       </c>
       <c r="E30" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A31" t="s">
-        <v>134</v>
-      </c>
-      <c r="C31">
-        <v>15</v>
-      </c>
-      <c r="D31" t="s">
-        <v>147</v>
-      </c>
-      <c r="E31" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A31" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3">
+        <v>11</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C32">
         <v>12</v>
@@ -1600,15 +1601,15 @@
         <v>152</v>
       </c>
       <c r="E32" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>91</v>
+        <v>123</v>
       </c>
       <c r="C33">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D33" t="s">
         <v>152</v>
@@ -1617,395 +1618,405 @@
         <v>156</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
+        <v>127</v>
+      </c>
+      <c r="C34">
+        <v>12</v>
+      </c>
+      <c r="D34" t="s">
+        <v>147</v>
+      </c>
+      <c r="E34" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
+        <v>125</v>
+      </c>
+      <c r="C35">
+        <v>12</v>
+      </c>
+      <c r="D35" t="s">
+        <v>147</v>
+      </c>
+      <c r="E35" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A36" t="s">
+        <v>124</v>
+      </c>
+      <c r="C36">
+        <v>12</v>
+      </c>
+      <c r="D36" t="s">
+        <v>147</v>
+      </c>
+      <c r="E36" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
+        <v>129</v>
+      </c>
+      <c r="C37">
+        <v>13</v>
+      </c>
+      <c r="D37" t="s">
+        <v>148</v>
+      </c>
+      <c r="E37" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A38" t="s">
+        <v>130</v>
+      </c>
+      <c r="C38">
+        <v>13</v>
+      </c>
+      <c r="D38" t="s">
+        <v>148</v>
+      </c>
+      <c r="E38" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A39" t="s">
         <v>128</v>
       </c>
-      <c r="C34">
+      <c r="C39">
         <v>13</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D39" t="s">
         <v>149</v>
-      </c>
-      <c r="E34" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
-        <v>114</v>
-      </c>
-      <c r="C35">
-        <v>8</v>
-      </c>
-      <c r="D35" t="s">
-        <v>149</v>
-      </c>
-      <c r="E35" t="s">
-        <v>156</v>
-      </c>
-      <c r="F35" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A36" t="s">
-        <v>88</v>
-      </c>
-      <c r="C36">
-        <v>2</v>
-      </c>
-      <c r="D36" t="s">
-        <v>149</v>
-      </c>
-      <c r="E36" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A37" t="s">
-        <v>90</v>
-      </c>
-      <c r="C37">
-        <v>2</v>
-      </c>
-      <c r="D37" t="s">
-        <v>149</v>
-      </c>
-      <c r="E37" t="s">
-        <v>156</v>
-      </c>
-      <c r="F37" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A38" t="s">
-        <v>140</v>
-      </c>
-      <c r="C38" t="s">
-        <v>143</v>
-      </c>
-      <c r="D38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E38" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A39" t="s">
-        <v>78</v>
-      </c>
-      <c r="B39">
-        <v>11</v>
-      </c>
-      <c r="D39" t="s">
-        <v>153</v>
       </c>
       <c r="E39" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>61</v>
-      </c>
-      <c r="B40">
-        <v>6</v>
+        <v>144</v>
+      </c>
+      <c r="C40">
+        <v>13</v>
       </c>
       <c r="D40" t="s">
+        <v>147</v>
+      </c>
+      <c r="E40" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A41" t="s">
+        <v>131</v>
+      </c>
+      <c r="C41">
+        <v>13</v>
+      </c>
+      <c r="D41" t="s">
+        <v>147</v>
+      </c>
+      <c r="E41" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A42" t="s">
+        <v>79</v>
+      </c>
+      <c r="B42">
+        <v>9</v>
+      </c>
+      <c r="C42">
+        <v>13</v>
+      </c>
+      <c r="D42" t="s">
+        <v>147</v>
+      </c>
+      <c r="E42" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A43" t="s">
+        <v>138</v>
+      </c>
+      <c r="C43">
+        <v>15</v>
+      </c>
+      <c r="D43" t="s">
         <v>152</v>
-      </c>
-      <c r="E40" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A41" t="s">
-        <v>138</v>
-      </c>
-      <c r="C41">
-        <v>15</v>
-      </c>
-      <c r="D41" t="s">
-        <v>152</v>
-      </c>
-      <c r="E41" t="s">
-        <v>158</v>
-      </c>
-      <c r="F41" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A42" t="s">
-        <v>95</v>
-      </c>
-      <c r="C42">
-        <v>4</v>
-      </c>
-      <c r="D42" t="s">
-        <v>149</v>
-      </c>
-      <c r="E42" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A43" t="s">
-        <v>85</v>
-      </c>
-      <c r="B43" t="s">
-        <v>80</v>
-      </c>
-      <c r="C43" t="s">
-        <v>145</v>
-      </c>
-      <c r="D43" t="s">
-        <v>149</v>
       </c>
       <c r="E43" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F43" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C44">
         <v>15</v>
       </c>
       <c r="D44" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E44" t="s">
+        <v>155</v>
+      </c>
+      <c r="F44" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="C45">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D45" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E45" t="s">
+        <v>155</v>
+      </c>
+      <c r="F45" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G45" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>63</v>
-      </c>
-      <c r="B46">
-        <v>7</v>
+        <v>133</v>
+      </c>
+      <c r="C46">
+        <v>15</v>
       </c>
       <c r="D46" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E46" t="s">
+        <v>155</v>
+      </c>
+      <c r="F46" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G46" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C47">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D47" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E47" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.45">
+        <v>157</v>
+      </c>
+      <c r="F47" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
-        <v>52</v>
-      </c>
-      <c r="B48" t="s">
-        <v>82</v>
+        <v>134</v>
+      </c>
+      <c r="C48">
+        <v>15</v>
       </c>
       <c r="D48" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E48" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>44</v>
-      </c>
-      <c r="B49">
-        <v>1</v>
+        <v>132</v>
+      </c>
+      <c r="C49">
+        <v>15</v>
       </c>
       <c r="D49" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E49" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>49</v>
-      </c>
-      <c r="B50">
-        <v>1</v>
+        <v>135</v>
+      </c>
+      <c r="C50">
+        <v>15</v>
       </c>
       <c r="D50" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="E50" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>67</v>
-      </c>
-      <c r="B51">
-        <v>8</v>
+        <v>85</v>
+      </c>
+      <c r="B51" t="s">
+        <v>80</v>
+      </c>
+      <c r="C51" t="s">
+        <v>145</v>
       </c>
       <c r="D51" t="s">
         <v>149</v>
       </c>
       <c r="E51" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A52" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B52" s="3"/>
+      <c r="C52" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E52" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="F51" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A52" t="s">
-        <v>131</v>
-      </c>
-      <c r="C52">
-        <v>13</v>
-      </c>
-      <c r="D52" t="s">
-        <v>147</v>
-      </c>
-      <c r="E52" t="s">
-        <v>154</v>
+      <c r="F52" s="3" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>48</v>
-      </c>
-      <c r="B53">
-        <v>1</v>
+        <v>119</v>
+      </c>
+      <c r="C53" t="s">
+        <v>146</v>
       </c>
       <c r="D53" t="s">
         <v>147</v>
       </c>
       <c r="E53" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A54" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="B54" s="3"/>
-      <c r="C54" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E54" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="F54" s="3" t="s">
+      <c r="A54" t="s">
+        <v>140</v>
+      </c>
+      <c r="C54" t="s">
+        <v>143</v>
+      </c>
+      <c r="D54" t="s">
+        <v>149</v>
+      </c>
+      <c r="E54" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A55" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B55" s="3"/>
+      <c r="C55" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E55" s="3" t="s">
         <v>163</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A55" t="s">
-        <v>79</v>
-      </c>
-      <c r="B55">
-        <v>9</v>
-      </c>
-      <c r="C55">
-        <v>13</v>
-      </c>
-      <c r="D55" t="s">
-        <v>147</v>
-      </c>
-      <c r="E55" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B56">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D56" t="s">
         <v>148</v>
       </c>
       <c r="E56" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B57">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D57" t="s">
         <v>148</v>
       </c>
       <c r="E57" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>122</v>
-      </c>
-      <c r="C58">
+        <v>77</v>
+      </c>
+      <c r="B58">
         <v>11</v>
       </c>
       <c r="D58" t="s">
         <v>148</v>
       </c>
       <c r="E58" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
-        <v>129</v>
-      </c>
-      <c r="C59">
-        <v>13</v>
+        <v>56</v>
+      </c>
+      <c r="B59">
+        <v>5</v>
       </c>
       <c r="D59" t="s">
         <v>148</v>
       </c>
       <c r="E59" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B60">
         <v>1</v>
@@ -2014,114 +2025,105 @@
         <v>148</v>
       </c>
       <c r="E60" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
-        <v>116</v>
-      </c>
-      <c r="C61">
-        <v>9</v>
+        <v>59</v>
+      </c>
+      <c r="B61">
+        <v>6</v>
       </c>
       <c r="D61" t="s">
         <v>148</v>
       </c>
       <c r="E61" t="s">
-        <v>157</v>
-      </c>
-      <c r="F61" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A62" t="s">
-        <v>130</v>
-      </c>
-      <c r="C62">
-        <v>13</v>
+      <c r="A62" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B62">
+        <v>5</v>
       </c>
       <c r="D62" t="s">
         <v>148</v>
       </c>
       <c r="E62" t="s">
-        <v>157</v>
+        <v>155</v>
+      </c>
+      <c r="F62" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
-        <v>66</v>
-      </c>
-      <c r="B63">
-        <v>8</v>
+        <v>52</v>
+      </c>
+      <c r="B63" t="s">
+        <v>82</v>
       </c>
       <c r="D63" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="E63" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B64">
         <v>1</v>
       </c>
       <c r="D64" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="E64" t="s">
-        <v>157</v>
-      </c>
-      <c r="F64" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>136</v>
-      </c>
-      <c r="C65">
-        <v>15</v>
+        <v>81</v>
+      </c>
+      <c r="B65">
+        <v>11</v>
       </c>
       <c r="D65" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E65" t="s">
         <v>157</v>
       </c>
-      <c r="F65" t="s">
-        <v>160</v>
-      </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>87</v>
-      </c>
-      <c r="C66">
-        <v>2</v>
+        <v>74</v>
+      </c>
+      <c r="B66">
+        <v>15</v>
       </c>
       <c r="D66" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E66" t="s">
         <v>157</v>
       </c>
-      <c r="F66" t="s">
-        <v>160</v>
-      </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
-        <v>169</v>
+        <v>46</v>
       </c>
       <c r="B67">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="D67" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E67" t="s">
         <v>157</v>
@@ -2129,92 +2131,83 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B68">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D68" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E68" t="s">
-        <v>157</v>
-      </c>
-      <c r="F68" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="B69">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D69" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E69" t="s">
-        <v>157</v>
-      </c>
-      <c r="F69" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B70">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D70" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E70" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B71">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D71" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E71" t="s">
-        <v>157</v>
-      </c>
-      <c r="F71" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="B72">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D72" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E72" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
-        <v>120</v>
-      </c>
-      <c r="C73">
-        <v>11</v>
+        <v>66</v>
+      </c>
+      <c r="B73">
+        <v>8</v>
       </c>
       <c r="D73" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E73" t="s">
         <v>157</v>
@@ -2222,247 +2215,255 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B74">
         <v>1</v>
       </c>
       <c r="D74" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E74" t="s">
         <v>157</v>
       </c>
+      <c r="F74" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
-        <v>93</v>
-      </c>
-      <c r="C75">
-        <v>2</v>
+        <v>68</v>
+      </c>
+      <c r="B75">
+        <v>8</v>
       </c>
       <c r="D75" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E75" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
-        <v>92</v>
-      </c>
-      <c r="C76">
+        <v>51</v>
+      </c>
+      <c r="B76">
         <v>2</v>
       </c>
       <c r="D76" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E76" t="s">
-        <v>157</v>
+        <v>155</v>
+      </c>
+      <c r="F76" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
-        <v>112</v>
-      </c>
-      <c r="C77">
+        <v>67</v>
+      </c>
+      <c r="B77">
         <v>8</v>
       </c>
       <c r="D77" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E77" t="s">
-        <v>168</v>
+        <v>154</v>
+      </c>
+      <c r="F77" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
-        <v>41</v>
+        <v>169</v>
       </c>
       <c r="B78">
-        <v>1</v>
-      </c>
-      <c r="C78">
+        <v>13</v>
+      </c>
+      <c r="D78" t="s">
+        <v>149</v>
+      </c>
+      <c r="E78" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A79" t="s">
+        <v>78</v>
+      </c>
+      <c r="B79">
         <v>11</v>
       </c>
-      <c r="D78" t="s">
-        <v>148</v>
-      </c>
-      <c r="E78" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A79" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="B79" s="3"/>
-      <c r="C79" s="3">
-        <v>6</v>
-      </c>
-      <c r="D79" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E79" s="3" t="s">
-        <v>168</v>
+      <c r="D79" t="s">
+        <v>153</v>
+      </c>
+      <c r="E79" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A80" t="s">
-        <v>68</v>
+      <c r="A80" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="B80">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D80" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E80" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A81" s="2" t="s">
-        <v>58</v>
+      <c r="A81" t="s">
+        <v>64</v>
       </c>
       <c r="B81">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D81" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="E81" t="s">
-        <v>168</v>
+        <v>155</v>
+      </c>
+      <c r="F81" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B82">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D82" t="s">
         <v>147</v>
       </c>
       <c r="E82" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
-        <v>38</v>
-      </c>
-      <c r="C83">
-        <v>5</v>
+        <v>48</v>
+      </c>
+      <c r="B83">
+        <v>1</v>
       </c>
       <c r="D83" t="s">
         <v>147</v>
       </c>
       <c r="E83" t="s">
-        <v>168</v>
-      </c>
-      <c r="F83" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="B84">
+        <v>4</v>
+      </c>
+      <c r="D84" t="s">
+        <v>147</v>
+      </c>
+      <c r="E84" t="s">
+        <v>157</v>
+      </c>
+      <c r="F84" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A85" t="s">
+        <v>42</v>
+      </c>
+      <c r="B85">
         <v>1</v>
       </c>
-      <c r="D84" t="s">
-        <v>147</v>
-      </c>
-      <c r="E84" t="s">
+      <c r="D85" t="s">
+        <v>147</v>
+      </c>
+      <c r="E85" t="s">
+        <v>157</v>
+      </c>
+      <c r="F85" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A85" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="B85" s="3"/>
-      <c r="C85" s="3">
-        <v>6</v>
-      </c>
-      <c r="D85" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E85" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A86" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3">
-        <v>11</v>
-      </c>
-      <c r="D86" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E86" s="3" t="s">
-        <v>168</v>
+      <c r="A86" t="s">
+        <v>54</v>
+      </c>
+      <c r="B86">
+        <v>4</v>
+      </c>
+      <c r="D86" t="s">
+        <v>147</v>
+      </c>
+      <c r="E86" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
-        <v>135</v>
-      </c>
-      <c r="C87">
-        <v>15</v>
+        <v>55</v>
+      </c>
+      <c r="B87">
+        <v>4</v>
       </c>
       <c r="D87" t="s">
         <v>147</v>
       </c>
       <c r="E87" t="s">
+        <v>157</v>
+      </c>
+      <c r="F87" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A88" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B88" s="3"/>
-      <c r="C88" s="3">
-        <v>4</v>
-      </c>
-      <c r="D88" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E88" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="F88" s="3" t="s">
-        <v>154</v>
+      <c r="A88" t="s">
+        <v>60</v>
+      </c>
+      <c r="B88">
+        <v>6</v>
+      </c>
+      <c r="D88" t="s">
+        <v>147</v>
+      </c>
+      <c r="E88" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
-        <v>125</v>
-      </c>
-      <c r="C89">
-        <v>12</v>
+        <v>47</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
       </c>
       <c r="D89" t="s">
         <v>147</v>
       </c>
       <c r="E89" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
-        <v>84</v>
-      </c>
-      <c r="B90" t="s">
-        <v>83</v>
+        <v>62</v>
+      </c>
+      <c r="B90">
+        <v>6</v>
       </c>
       <c r="D90" t="s">
         <v>147</v>
@@ -2470,19 +2471,13 @@
       <c r="E90" t="s">
         <v>168</v>
       </c>
-      <c r="F90" t="s">
-        <v>163</v>
-      </c>
-      <c r="G90" t="s">
-        <v>164</v>
-      </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
-        <v>124</v>
-      </c>
-      <c r="C91">
-        <v>12</v>
+        <v>39</v>
+      </c>
+      <c r="B91">
+        <v>1</v>
       </c>
       <c r="D91" t="s">
         <v>147</v>
@@ -2492,37 +2487,42 @@
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A92" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B92" s="3"/>
-      <c r="C92" s="3">
-        <v>6</v>
-      </c>
-      <c r="D92" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E92" s="3" t="s">
+      <c r="A92" t="s">
+        <v>84</v>
+      </c>
+      <c r="B92" t="s">
+        <v>83</v>
+      </c>
+      <c r="D92" t="s">
+        <v>147</v>
+      </c>
+      <c r="E92" t="s">
         <v>168</v>
+      </c>
+      <c r="F92" t="s">
+        <v>163</v>
+      </c>
+      <c r="G92" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
-        <v>165</v>
-      </c>
-      <c r="C93">
-        <v>9</v>
+        <v>40</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
       </c>
       <c r="D93" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="E93" t="s">
-        <v>167</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G92">
-    <sortCondition ref="E2:E92"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G93">
+    <sortCondition ref="C2:C93"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add stuff to draf
</commit_message>
<xml_diff>
--- a/Research/TheProjectKaggle/leaderboardanalysis/Topgold/Whatworkeddidntwork.xlsx
+++ b/Research/TheProjectKaggle/leaderboardanalysis/Topgold/Whatworkeddidntwork.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shwes\Projects\Thesis\Research\TheProjectKaggle\leaderboardanalysis\Topgold\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24BB4C1C-AB94-4FB2-BA55-C3CEDB965EE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B17A5D24-74C5-47CD-8289-E209E3300C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Place Focused" sheetId="1" r:id="rId1"/>
@@ -549,7 +549,7 @@
     <t>more complicated Training Technique did not help as much as better data and preprocessing</t>
   </si>
   <si>
-    <t xml:space="preserve">ensembled a ByT5-Large and a ByT5-XL model, using a fine-tuned Qwen3-8B pairwise Reward Model to select the better translation per sentence, </t>
+    <t>ensembled a ByT5-Large and a ByT5-XL model, using a fine-tuned Qwen3-8B pairwise Reward Model to select the better translation per sentence, used Claude 4.5 Sonnet to generate diverse synthetic tasks to teach Old Akkadian fundamentals to ByT5 models., extracting lemmas from dictionaries and making synthetic data from them, using grammar rules with an LLM to hand construct sentences.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Add 3rd place what worked
</commit_message>
<xml_diff>
--- a/Research/TheProjectKaggle/leaderboardanalysis/Topgold/Whatworkeddidntwork.xlsx
+++ b/Research/TheProjectKaggle/leaderboardanalysis/Topgold/Whatworkeddidntwork.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shwes\Projects\Thesis\Research\TheProjectKaggle\leaderboardanalysis\Topgold\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B17A5D24-74C5-47CD-8289-E209E3300C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148173B8-0FBA-4F50-967F-9CF06F26A4B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Place Focused" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="178">
   <si>
     <t>Placement</t>
   </si>
@@ -549,7 +549,28 @@
     <t>more complicated Training Technique did not help as much as better data and preprocessing</t>
   </si>
   <si>
-    <t>ensembled a ByT5-Large and a ByT5-XL model, using a fine-tuned Qwen3-8B pairwise Reward Model to select the better translation per sentence, used Claude 4.5 Sonnet to generate diverse synthetic tasks to teach Old Akkadian fundamentals to ByT5 models., extracting lemmas from dictionaries and making synthetic data from them, using grammar rules with an LLM to hand construct sentences.</t>
+    <t xml:space="preserve">ensembled a ByT5-Large and a ByT5-XL model, </t>
+  </si>
+  <si>
+    <t>using a fine-tuned Qwen3-8B pairwise Reward Model to select the better translation per sentence</t>
+  </si>
+  <si>
+    <t>used Claude 4.5 Sonnet to generate diverse synthetic tasks to teach Old Akkadian fundamentals to ByT5 models</t>
+  </si>
+  <si>
+    <t>extracting lemmas from dictionaries and making synthetic data from them</t>
+  </si>
+  <si>
+    <t>using grammar rules with an LLM to hand construct sentences</t>
+  </si>
+  <si>
+    <t>ensembled a ByT5-Large and a ByT5-XL model, using a fine-tuned Qwen3-8B pairwise Reward Model to select the better translation per sentence, used Claude 4.5 Sonnet to generate diverse synthetic tasks to teach Old Akkadian fundamentals to ByT5 models., extracting lemmas from dictionaries and making synthetic data from them, using grammar rules with an LLM to hand construct sentences., Gemini pro for text extraction, beam search with 8 beams.</t>
+  </si>
+  <si>
+    <t>Gemini pro for text extraction</t>
+  </si>
+  <si>
+    <t>Beam search with 8 beams.</t>
   </si>
 </sst>
 </file>
@@ -962,7 +983,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -1102,7 +1123,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59139DE4-7389-4BBE-B315-1A18956BA69C}">
-  <dimension ref="A1:G93"/>
+  <dimension ref="A1:G100"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="64.86328125" customWidth="1"/>
@@ -1153,166 +1174,154 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="E3" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="C4">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E4" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C5">
-        <v>2</v>
-      </c>
-      <c r="D5" t="s">
-        <v>149</v>
-      </c>
-      <c r="E5" t="s">
-        <v>156</v>
-      </c>
-      <c r="F5" t="s">
-        <v>168</v>
+      <c r="A5" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3">
+        <v>6</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>87</v>
+        <v>113</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E6" t="s">
-        <v>157</v>
-      </c>
-      <c r="F6" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>93</v>
+        <v>144</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
         <v>147</v>
       </c>
       <c r="E7" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>92</v>
-      </c>
-      <c r="C8">
-        <v>2</v>
+        <v>75</v>
+      </c>
+      <c r="B8">
+        <v>9</v>
       </c>
       <c r="D8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E8" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>95</v>
-      </c>
-      <c r="C9">
-        <v>4</v>
+        <v>76</v>
+      </c>
+      <c r="B9">
+        <v>9</v>
       </c>
       <c r="D9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E9" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>96</v>
-      </c>
-      <c r="C10">
-        <v>4</v>
+        <v>77</v>
+      </c>
+      <c r="B10">
+        <v>11</v>
       </c>
       <c r="D10" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E10" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A11" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3">
-        <v>4</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>154</v>
+      <c r="A11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>148</v>
+      </c>
+      <c r="E11" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12">
-        <v>5</v>
+        <v>43</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
       </c>
       <c r="D12" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E12" t="s">
-        <v>168</v>
-      </c>
-      <c r="F12" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>108</v>
-      </c>
-      <c r="C13">
-        <v>6</v>
+        <v>40</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E13" t="s">
         <v>148</v>
@@ -1320,740 +1329,762 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="C14">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s">
+        <v>149</v>
+      </c>
+      <c r="E14" t="s">
+        <v>155</v>
+      </c>
+      <c r="F14" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="D15" t="s">
+        <v>149</v>
+      </c>
+      <c r="E15" t="s">
+        <v>155</v>
+      </c>
+      <c r="F15" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16">
+        <v>8</v>
+      </c>
+      <c r="D16" t="s">
+        <v>147</v>
+      </c>
+      <c r="E16" t="s">
+        <v>155</v>
+      </c>
+      <c r="F16" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>139</v>
+      </c>
+      <c r="B17"/>
+      <c r="C17">
+        <v>15</v>
+      </c>
+      <c r="D17" t="s">
+        <v>149</v>
+      </c>
+      <c r="E17" t="s">
+        <v>155</v>
+      </c>
+      <c r="F17" t="s">
+        <v>158</v>
+      </c>
+      <c r="G17" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>133</v>
+      </c>
+      <c r="C18">
+        <v>15</v>
+      </c>
+      <c r="D18" t="s">
+        <v>149</v>
+      </c>
+      <c r="E18" t="s">
+        <v>155</v>
+      </c>
+      <c r="F18" t="s">
+        <v>158</v>
+      </c>
+      <c r="G18" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>137</v>
+      </c>
+      <c r="C19">
+        <v>15</v>
+      </c>
+      <c r="D19" t="s">
+        <v>149</v>
+      </c>
+      <c r="E19" t="s">
+        <v>155</v>
+      </c>
+      <c r="F19" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A20" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B20">
+        <v>5</v>
+      </c>
+      <c r="D20" t="s">
+        <v>148</v>
+      </c>
+      <c r="E20" t="s">
+        <v>155</v>
+      </c>
+      <c r="F20" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>126</v>
+      </c>
+      <c r="C21">
+        <v>12</v>
+      </c>
+      <c r="D21" t="s">
+        <v>152</v>
+      </c>
+      <c r="E21" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22">
         <v>6</v>
       </c>
-      <c r="D14" t="s">
-        <v>148</v>
-      </c>
-      <c r="E14" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A15" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3">
+      <c r="D22" t="s">
+        <v>148</v>
+      </c>
+      <c r="E22" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>65</v>
+      </c>
+      <c r="B23">
+        <v>8</v>
+      </c>
+      <c r="D23" t="s">
+        <v>152</v>
+      </c>
+      <c r="E23" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24">
+        <v>15</v>
+      </c>
+      <c r="D24" t="s">
+        <v>152</v>
+      </c>
+      <c r="E24" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="D25" t="s">
+        <v>152</v>
+      </c>
+      <c r="E25" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>96</v>
+      </c>
+      <c r="C26">
+        <v>4</v>
+      </c>
+      <c r="D26" t="s">
+        <v>147</v>
+      </c>
+      <c r="E26" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A27" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B27" s="3">
+        <v>8</v>
+      </c>
+      <c r="C27" s="3">
         <v>6</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A16" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3">
-        <v>6</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B17" s="3">
+      <c r="D27" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>115</v>
+      </c>
+      <c r="C28">
+        <v>9</v>
+      </c>
+      <c r="D28" t="s">
+        <v>147</v>
+      </c>
+      <c r="E28" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A29" t="s">
+        <v>134</v>
+      </c>
+      <c r="C29">
+        <v>15</v>
+      </c>
+      <c r="D29" t="s">
+        <v>147</v>
+      </c>
+      <c r="E29" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A30" t="s">
+        <v>119</v>
+      </c>
+      <c r="C30" t="s">
+        <v>146</v>
+      </c>
+      <c r="D30" t="s">
+        <v>147</v>
+      </c>
+      <c r="E30" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A31" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A32" t="s">
+        <v>114</v>
+      </c>
+      <c r="C32">
         <v>8</v>
       </c>
-      <c r="C17" s="3">
-        <v>6</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A18" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3">
-        <v>6</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A19" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3">
-        <v>6</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
-        <v>113</v>
-      </c>
-      <c r="C20">
-        <v>8</v>
-      </c>
-      <c r="D20" t="s">
-        <v>148</v>
-      </c>
-      <c r="E20" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
-        <v>112</v>
-      </c>
-      <c r="C21">
-        <v>8</v>
-      </c>
-      <c r="D21" t="s">
-        <v>148</v>
-      </c>
-      <c r="E21" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
-        <v>114</v>
-      </c>
-      <c r="C22">
-        <v>8</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="D32" t="s">
         <v>149</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E32" t="s">
         <v>156</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F32" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A23" t="s">
-        <v>116</v>
-      </c>
-      <c r="C23">
-        <v>9</v>
-      </c>
-      <c r="D23" t="s">
-        <v>148</v>
-      </c>
-      <c r="E23" t="s">
-        <v>157</v>
-      </c>
-      <c r="F23" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
-        <v>115</v>
-      </c>
-      <c r="C24">
-        <v>9</v>
-      </c>
-      <c r="D24" t="s">
-        <v>147</v>
-      </c>
-      <c r="E24" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A25" t="s">
-        <v>165</v>
-      </c>
-      <c r="C25">
-        <v>9</v>
-      </c>
-      <c r="D25" t="s">
-        <v>147</v>
-      </c>
-      <c r="E25" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A26" t="s">
-        <v>117</v>
-      </c>
-      <c r="C26">
-        <v>9</v>
-      </c>
-      <c r="D26" t="s">
-        <v>151</v>
-      </c>
-      <c r="E26" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A27" t="s">
-        <v>122</v>
-      </c>
-      <c r="C27">
-        <v>11</v>
-      </c>
-      <c r="D27" t="s">
-        <v>148</v>
-      </c>
-      <c r="E27" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A28" t="s">
-        <v>41</v>
-      </c>
-      <c r="B28">
-        <v>1</v>
-      </c>
-      <c r="C28">
-        <v>11</v>
-      </c>
-      <c r="D28" t="s">
-        <v>148</v>
-      </c>
-      <c r="E28" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A29" t="s">
-        <v>121</v>
-      </c>
-      <c r="C29">
-        <v>11</v>
-      </c>
-      <c r="D29" t="s">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
+        <v>90</v>
+      </c>
+      <c r="C33">
+        <v>2</v>
+      </c>
+      <c r="D33" t="s">
         <v>149</v>
-      </c>
-      <c r="E29" t="s">
-        <v>155</v>
-      </c>
-      <c r="F29" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A30" t="s">
-        <v>120</v>
-      </c>
-      <c r="C30">
-        <v>11</v>
-      </c>
-      <c r="D30" t="s">
-        <v>147</v>
-      </c>
-      <c r="E30" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A31" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3">
-        <v>11</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A32" t="s">
-        <v>126</v>
-      </c>
-      <c r="C32">
-        <v>12</v>
-      </c>
-      <c r="D32" t="s">
-        <v>152</v>
-      </c>
-      <c r="E32" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A33" t="s">
-        <v>123</v>
-      </c>
-      <c r="C33">
-        <v>12</v>
-      </c>
-      <c r="D33" t="s">
-        <v>152</v>
       </c>
       <c r="E33" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="F33" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>127</v>
+        <v>91</v>
       </c>
       <c r="C34">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D34" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E34" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>125</v>
+        <v>88</v>
       </c>
       <c r="C35">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D35" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E35" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C36">
         <v>12</v>
       </c>
       <c r="D36" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E36" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C37">
         <v>13</v>
       </c>
       <c r="D37" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E37" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>130</v>
-      </c>
-      <c r="C38">
-        <v>13</v>
+        <v>140</v>
+      </c>
+      <c r="C38" t="s">
+        <v>143</v>
       </c>
       <c r="D38" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E38" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>128</v>
-      </c>
-      <c r="C39">
-        <v>13</v>
+        <v>78</v>
+      </c>
+      <c r="B39">
+        <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="E39" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C40">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D40" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E40" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+        <v>158</v>
+      </c>
+      <c r="F40" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>131</v>
+        <v>95</v>
       </c>
       <c r="C41">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D41" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E41" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
-        <v>79</v>
-      </c>
-      <c r="B42">
+        <v>117</v>
+      </c>
+      <c r="C42">
         <v>9</v>
       </c>
-      <c r="C42">
-        <v>13</v>
-      </c>
       <c r="D42" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="E42" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="C43">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D43" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="E43" t="s">
         <v>158</v>
       </c>
-      <c r="F43" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C44">
         <v>15</v>
       </c>
       <c r="D44" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E44" t="s">
-        <v>155</v>
-      </c>
-      <c r="F44" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>139</v>
-      </c>
-      <c r="C45">
-        <v>15</v>
+        <v>85</v>
+      </c>
+      <c r="B45" t="s">
+        <v>80</v>
+      </c>
+      <c r="C45" t="s">
+        <v>145</v>
       </c>
       <c r="D45" t="s">
         <v>149</v>
       </c>
       <c r="E45" t="s">
-        <v>155</v>
-      </c>
-      <c r="F45" t="s">
         <v>158</v>
       </c>
-      <c r="G45" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>133</v>
-      </c>
-      <c r="C46">
-        <v>15</v>
+        <v>61</v>
+      </c>
+      <c r="B46">
+        <v>6</v>
       </c>
       <c r="D46" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E46" t="s">
-        <v>155</v>
-      </c>
-      <c r="F46" t="s">
         <v>158</v>
       </c>
-      <c r="G46" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>136</v>
-      </c>
-      <c r="C47">
-        <v>15</v>
+        <v>63</v>
+      </c>
+      <c r="B47">
+        <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E47" t="s">
-        <v>157</v>
-      </c>
-      <c r="F47" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A48" t="s">
-        <v>134</v>
-      </c>
-      <c r="C48">
-        <v>15</v>
-      </c>
-      <c r="D48" t="s">
-        <v>147</v>
-      </c>
-      <c r="E48" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A48" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B48" s="3"/>
+      <c r="C48" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="F48" s="3" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>132</v>
-      </c>
-      <c r="C49">
-        <v>15</v>
+        <v>67</v>
+      </c>
+      <c r="B49">
+        <v>8</v>
       </c>
       <c r="D49" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E49" t="s">
-        <v>158</v>
+        <v>154</v>
+      </c>
+      <c r="F49" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C50">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D50" t="s">
         <v>147</v>
       </c>
       <c r="E50" t="s">
-        <v>168</v>
+        <v>154</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>85</v>
-      </c>
-      <c r="B51" t="s">
-        <v>80</v>
-      </c>
-      <c r="C51" t="s">
-        <v>145</v>
+        <v>79</v>
+      </c>
+      <c r="B51">
+        <v>9</v>
+      </c>
+      <c r="C51">
+        <v>13</v>
       </c>
       <c r="D51" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E51" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A52" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="B52" s="3"/>
-      <c r="C52" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="D52" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E52" s="3" t="s">
+      <c r="A52" t="s">
+        <v>52</v>
+      </c>
+      <c r="B52" t="s">
+        <v>82</v>
+      </c>
+      <c r="D52" t="s">
+        <v>148</v>
+      </c>
+      <c r="E52" t="s">
         <v>154</v>
-      </c>
-      <c r="F52" s="3" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>119</v>
-      </c>
-      <c r="C53" t="s">
-        <v>146</v>
+        <v>44</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
       </c>
       <c r="D53" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E53" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
-        <v>140</v>
-      </c>
-      <c r="C54" t="s">
-        <v>143</v>
+        <v>49</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
       </c>
       <c r="D54" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E54" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A55" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B55" s="3"/>
-      <c r="C55" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="D55" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>163</v>
+      <c r="A55" t="s">
+        <v>48</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="D55" t="s">
+        <v>147</v>
+      </c>
+      <c r="E55" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>75</v>
-      </c>
-      <c r="B56">
+        <v>116</v>
+      </c>
+      <c r="C56">
         <v>9</v>
       </c>
       <c r="D56" t="s">
         <v>148</v>
       </c>
       <c r="E56" t="s">
-        <v>148</v>
+        <v>157</v>
+      </c>
+      <c r="F56" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>76</v>
-      </c>
-      <c r="B57">
-        <v>9</v>
+        <v>87</v>
+      </c>
+      <c r="C57">
+        <v>2</v>
       </c>
       <c r="D57" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E57" t="s">
-        <v>148</v>
+        <v>157</v>
+      </c>
+      <c r="F57" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>77</v>
-      </c>
-      <c r="B58">
-        <v>11</v>
+        <v>136</v>
+      </c>
+      <c r="C58">
+        <v>15</v>
       </c>
       <c r="D58" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E58" t="s">
-        <v>148</v>
+        <v>157</v>
+      </c>
+      <c r="F58" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B59">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D59" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E59" t="s">
-        <v>148</v>
+        <v>157</v>
+      </c>
+      <c r="F59" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="B60">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D60" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E60" t="s">
-        <v>148</v>
+        <v>157</v>
+      </c>
+      <c r="F60" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="B61">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D61" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E61" t="s">
-        <v>155</v>
+        <v>157</v>
+      </c>
+      <c r="F61" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A62" s="2" t="s">
-        <v>57</v>
+      <c r="A62" t="s">
+        <v>55</v>
       </c>
       <c r="B62">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D62" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E62" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F62" t="s">
         <v>168</v>
@@ -2061,37 +2092,37 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
-        <v>52</v>
-      </c>
-      <c r="B63" t="s">
-        <v>82</v>
+        <v>93</v>
+      </c>
+      <c r="C63">
+        <v>2</v>
       </c>
       <c r="D63" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E63" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
-        <v>44</v>
-      </c>
-      <c r="B64">
-        <v>1</v>
+        <v>92</v>
+      </c>
+      <c r="C64">
+        <v>2</v>
       </c>
       <c r="D64" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E64" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>81</v>
-      </c>
-      <c r="B65">
+        <v>122</v>
+      </c>
+      <c r="C65">
         <v>11</v>
       </c>
       <c r="D65" t="s">
@@ -2101,26 +2132,26 @@
         <v>157</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>74</v>
-      </c>
-      <c r="B66">
-        <v>15</v>
+        <v>120</v>
+      </c>
+      <c r="C66">
+        <v>11</v>
       </c>
       <c r="D66" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E66" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
-        <v>46</v>
-      </c>
-      <c r="B67">
-        <v>1</v>
+        <v>129</v>
+      </c>
+      <c r="C67">
+        <v>13</v>
       </c>
       <c r="D67" t="s">
         <v>148</v>
@@ -2129,369 +2160,368 @@
         <v>157</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
-        <v>65</v>
-      </c>
-      <c r="B68">
+        <v>130</v>
+      </c>
+      <c r="C68">
+        <v>13</v>
+      </c>
+      <c r="D68" t="s">
+        <v>148</v>
+      </c>
+      <c r="E68" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A69" t="s">
+        <v>81</v>
+      </c>
+      <c r="B69">
+        <v>11</v>
+      </c>
+      <c r="D69" t="s">
+        <v>148</v>
+      </c>
+      <c r="E69" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A70" t="s">
+        <v>74</v>
+      </c>
+      <c r="B70">
+        <v>15</v>
+      </c>
+      <c r="D70" t="s">
+        <v>148</v>
+      </c>
+      <c r="E70" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A71" t="s">
+        <v>46</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="D71" t="s">
+        <v>148</v>
+      </c>
+      <c r="E71" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A72" t="s">
+        <v>66</v>
+      </c>
+      <c r="B72">
         <v>8</v>
-      </c>
-      <c r="D68" t="s">
-        <v>152</v>
-      </c>
-      <c r="E68" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A69" t="s">
-        <v>73</v>
-      </c>
-      <c r="B69">
-        <v>15</v>
-      </c>
-      <c r="D69" t="s">
-        <v>152</v>
-      </c>
-      <c r="E69" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A70" t="s">
-        <v>50</v>
-      </c>
-      <c r="B70">
-        <v>2</v>
-      </c>
-      <c r="D70" t="s">
-        <v>152</v>
-      </c>
-      <c r="E70" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A71" t="s">
-        <v>61</v>
-      </c>
-      <c r="B71">
-        <v>6</v>
-      </c>
-      <c r="D71" t="s">
-        <v>152</v>
-      </c>
-      <c r="E71" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A72" t="s">
-        <v>49</v>
-      </c>
-      <c r="B72">
-        <v>1</v>
       </c>
       <c r="D72" t="s">
         <v>152</v>
       </c>
       <c r="E72" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.45">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
-        <v>66</v>
+        <v>169</v>
       </c>
       <c r="B73">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D73" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E73" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="B74">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D74" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="E74" t="s">
         <v>157</v>
       </c>
-      <c r="F74" t="s">
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A75" t="s">
+        <v>60</v>
+      </c>
+      <c r="B75">
+        <v>6</v>
+      </c>
+      <c r="D75" t="s">
+        <v>147</v>
+      </c>
+      <c r="E75" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A76" t="s">
+        <v>47</v>
+      </c>
+      <c r="B76">
+        <v>1</v>
+      </c>
+      <c r="D76" t="s">
+        <v>147</v>
+      </c>
+      <c r="E76" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A77" t="s">
+        <v>165</v>
+      </c>
+      <c r="C77">
+        <v>9</v>
+      </c>
+      <c r="D77" t="s">
+        <v>147</v>
+      </c>
+      <c r="E77" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A78" t="s">
+        <v>38</v>
+      </c>
+      <c r="C78">
+        <v>5</v>
+      </c>
+      <c r="D78" t="s">
+        <v>147</v>
+      </c>
+      <c r="E78" t="s">
+        <v>168</v>
+      </c>
+      <c r="F78" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A79" t="s">
+        <v>84</v>
+      </c>
+      <c r="B79" t="s">
+        <v>83</v>
+      </c>
+      <c r="D79" t="s">
+        <v>147</v>
+      </c>
+      <c r="E79" t="s">
+        <v>168</v>
+      </c>
+      <c r="F79" t="s">
+        <v>163</v>
+      </c>
+      <c r="G79" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A80" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B80" s="3"/>
+      <c r="C80" s="3">
+        <v>4</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E80" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F80" s="3" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A75" t="s">
-        <v>68</v>
-      </c>
-      <c r="B75">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A81" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81" s="3"/>
+      <c r="C81" s="3">
+        <v>6</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E81" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A82" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B82" s="3"/>
+      <c r="C82" s="3">
+        <v>6</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E82" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A83" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B83" s="3"/>
+      <c r="C83" s="3">
+        <v>6</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E83" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="C84">
         <v>8</v>
       </c>
-      <c r="D75" t="s">
-        <v>152</v>
-      </c>
-      <c r="E75" t="s">
+      <c r="D84" t="s">
+        <v>148</v>
+      </c>
+      <c r="E84" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A76" t="s">
-        <v>51</v>
-      </c>
-      <c r="B76">
-        <v>2</v>
-      </c>
-      <c r="D76" t="s">
-        <v>149</v>
-      </c>
-      <c r="E76" t="s">
-        <v>155</v>
-      </c>
-      <c r="F76" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A77" t="s">
-        <v>67</v>
-      </c>
-      <c r="B77">
-        <v>8</v>
-      </c>
-      <c r="D77" t="s">
-        <v>149</v>
-      </c>
-      <c r="E77" t="s">
-        <v>154</v>
-      </c>
-      <c r="F77" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A78" t="s">
-        <v>169</v>
-      </c>
-      <c r="B78">
-        <v>13</v>
-      </c>
-      <c r="D78" t="s">
-        <v>149</v>
-      </c>
-      <c r="E78" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A79" t="s">
-        <v>78</v>
-      </c>
-      <c r="B79">
-        <v>11</v>
-      </c>
-      <c r="D79" t="s">
-        <v>153</v>
-      </c>
-      <c r="E79" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A80" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B80">
-        <v>5</v>
-      </c>
-      <c r="D80" t="s">
-        <v>153</v>
-      </c>
-      <c r="E80" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A81" t="s">
-        <v>64</v>
-      </c>
-      <c r="B81">
-        <v>8</v>
-      </c>
-      <c r="D81" t="s">
-        <v>147</v>
-      </c>
-      <c r="E81" t="s">
-        <v>155</v>
-      </c>
-      <c r="F81" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A82" t="s">
-        <v>63</v>
-      </c>
-      <c r="B82">
-        <v>7</v>
-      </c>
-      <c r="D82" t="s">
-        <v>147</v>
-      </c>
-      <c r="E82" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A83" t="s">
-        <v>48</v>
-      </c>
-      <c r="B83">
-        <v>1</v>
-      </c>
-      <c r="D83" t="s">
-        <v>147</v>
-      </c>
-      <c r="E83" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A84" t="s">
-        <v>53</v>
-      </c>
-      <c r="B84">
-        <v>4</v>
-      </c>
-      <c r="D84" t="s">
-        <v>147</v>
-      </c>
-      <c r="E84" t="s">
-        <v>157</v>
-      </c>
-      <c r="F84" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B85">
         <v>1</v>
       </c>
+      <c r="C85">
+        <v>11</v>
+      </c>
       <c r="D85" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E85" t="s">
-        <v>157</v>
-      </c>
-      <c r="F85" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A86" t="s">
-        <v>54</v>
-      </c>
-      <c r="B86">
-        <v>4</v>
-      </c>
-      <c r="D86" t="s">
-        <v>147</v>
-      </c>
-      <c r="E86" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A86" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B86" s="3"/>
+      <c r="C86" s="3">
+        <v>11</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E86" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
-        <v>55</v>
-      </c>
-      <c r="B87">
-        <v>4</v>
+        <v>125</v>
+      </c>
+      <c r="C87">
+        <v>12</v>
       </c>
       <c r="D87" t="s">
         <v>147</v>
       </c>
       <c r="E87" t="s">
-        <v>157</v>
-      </c>
-      <c r="F87" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
-        <v>60</v>
-      </c>
-      <c r="B88">
-        <v>6</v>
+        <v>124</v>
+      </c>
+      <c r="C88">
+        <v>12</v>
       </c>
       <c r="D88" t="s">
         <v>147</v>
       </c>
       <c r="E88" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.45">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
-        <v>47</v>
-      </c>
-      <c r="B89">
-        <v>1</v>
+        <v>135</v>
+      </c>
+      <c r="C89">
+        <v>15</v>
       </c>
       <c r="D89" t="s">
         <v>147</v>
       </c>
       <c r="E89" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.45">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B90">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D90" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E90" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A91" t="s">
-        <v>39</v>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A91" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="B91">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D91" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E91" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
-        <v>84</v>
-      </c>
-      <c r="B92" t="s">
-        <v>83</v>
+        <v>62</v>
+      </c>
+      <c r="B92">
+        <v>6</v>
       </c>
       <c r="D92" t="s">
         <v>147</v>
@@ -2499,30 +2529,115 @@
       <c r="E92" t="s">
         <v>168</v>
       </c>
-      <c r="F92" t="s">
-        <v>163</v>
-      </c>
-      <c r="G92" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.45">
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B93">
         <v>1</v>
       </c>
       <c r="D93" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="E93" t="s">
-        <v>148</v>
+        <v>168</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A94" t="s">
+        <v>170</v>
+      </c>
+      <c r="C94">
+        <v>3</v>
+      </c>
+      <c r="E94" t="s">
+        <v>163</v>
+      </c>
+      <c r="F94" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A95" t="s">
+        <v>171</v>
+      </c>
+      <c r="C95">
+        <v>3</v>
+      </c>
+      <c r="E95" t="s">
+        <v>154</v>
+      </c>
+      <c r="F95" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A96" t="s">
+        <v>172</v>
+      </c>
+      <c r="C96">
+        <v>3</v>
+      </c>
+      <c r="E96" t="s">
+        <v>155</v>
+      </c>
+      <c r="F96" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A97" t="s">
+        <v>173</v>
+      </c>
+      <c r="C97">
+        <v>3</v>
+      </c>
+      <c r="E97" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A98" t="s">
+        <v>174</v>
+      </c>
+      <c r="C98">
+        <v>3</v>
+      </c>
+      <c r="E98" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A99" t="s">
+        <v>176</v>
+      </c>
+      <c r="C99">
+        <v>3</v>
+      </c>
+      <c r="E99" t="s">
+        <v>156</v>
+      </c>
+      <c r="F99" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A100" t="s">
+        <v>177</v>
+      </c>
+      <c r="C100">
+        <v>3</v>
+      </c>
+      <c r="E100" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G93">
-    <sortCondition ref="C2:C93"/>
+    <sortCondition ref="E2:E93"/>
+    <sortCondition ref="F2:F93"/>
+    <sortCondition ref="G2:G93"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Go through 1-15 to check future work
</commit_message>
<xml_diff>
--- a/Research/TheProjectKaggle/leaderboardanalysis/Topgold/Whatworkeddidntwork.xlsx
+++ b/Research/TheProjectKaggle/leaderboardanalysis/Topgold/Whatworkeddidntwork.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shwes\Projects\Thesis\Research\TheProjectKaggle\leaderboardanalysis\Topgold\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148173B8-0FBA-4F50-967F-9CF06F26A4B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{266B5028-EC26-40D3-A8C6-33C5BCD63664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Place Focused" sheetId="1" r:id="rId1"/>
-    <sheet name="Technique fixed" sheetId="4" r:id="rId2"/>
+    <sheet name="Key" sheetId="5" r:id="rId2"/>
+    <sheet name="Technique fixed" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="183">
   <si>
     <t>Placement</t>
   </si>
@@ -571,6 +572,21 @@
   </si>
   <si>
     <t>Beam search with 8 beams.</t>
+  </si>
+  <si>
+    <t>Did before kaggle ended</t>
+  </si>
+  <si>
+    <t>Did in my final testing</t>
+  </si>
+  <si>
+    <t>Want to do in my final testing</t>
+  </si>
+  <si>
+    <t>Hard but sounds fruitful</t>
+  </si>
+  <si>
+    <t>I'd rather copy</t>
   </si>
 </sst>
 </file>
@@ -606,7 +622,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -627,7 +643,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -644,12 +666,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1122,6 +1147,31 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47BA448A-A12C-425A-B034-D7C3798CDC09}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A1" s="7" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A2" s="5" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A3" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59139DE4-7389-4BBE-B315-1A18956BA69C}">
   <dimension ref="A1:G100"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1387,7 +1437,7 @@
         <v>15</v>
       </c>
       <c r="D17" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E17" t="s">
         <v>155</v>
@@ -1621,7 +1671,7 @@
         <v>8</v>
       </c>
       <c r="D32" t="s">
-        <v>149</v>
+        <v>182</v>
       </c>
       <c r="E32" t="s">
         <v>156</v>
@@ -1638,7 +1688,7 @@
         <v>2</v>
       </c>
       <c r="D33" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E33" t="s">
         <v>156</v>
@@ -1669,7 +1719,7 @@
         <v>2</v>
       </c>
       <c r="D35" t="s">
-        <v>149</v>
+        <v>182</v>
       </c>
       <c r="E35" t="s">
         <v>156</v>
@@ -1697,7 +1747,7 @@
         <v>13</v>
       </c>
       <c r="D37" t="s">
-        <v>149</v>
+        <v>182</v>
       </c>
       <c r="E37" t="s">
         <v>156</v>
@@ -1711,7 +1761,7 @@
         <v>143</v>
       </c>
       <c r="D38" t="s">
-        <v>149</v>
+        <v>182</v>
       </c>
       <c r="E38" t="s">
         <v>156</v>
@@ -2502,17 +2552,17 @@
         <v>168</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A91" s="2" t="s">
+    <row r="91" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A91" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B91">
+      <c r="B91" s="7">
         <v>5</v>
       </c>
-      <c r="D91" t="s">
+      <c r="D91" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="E91" t="s">
+      <c r="E91" s="7" t="s">
         <v>168</v>
       </c>
     </row>
@@ -2551,6 +2601,9 @@
       <c r="C94">
         <v>3</v>
       </c>
+      <c r="D94" t="s">
+        <v>149</v>
+      </c>
       <c r="E94" t="s">
         <v>163</v>
       </c>
@@ -2565,6 +2618,9 @@
       <c r="C95">
         <v>3</v>
       </c>
+      <c r="D95" t="s">
+        <v>152</v>
+      </c>
       <c r="E95" t="s">
         <v>154</v>
       </c>
@@ -2572,17 +2628,20 @@
         <v>158</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A96" t="s">
+    <row r="96" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A96" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="C96">
+      <c r="C96" s="3">
         <v>3</v>
       </c>
-      <c r="E96" t="s">
+      <c r="D96" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E96" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="F96" t="s">
+      <c r="F96" s="3" t="s">
         <v>168</v>
       </c>
     </row>
@@ -2593,6 +2652,9 @@
       <c r="C97">
         <v>3</v>
       </c>
+      <c r="D97" t="s">
+        <v>182</v>
+      </c>
       <c r="E97" t="s">
         <v>155</v>
       </c>
@@ -2604,6 +2666,9 @@
       <c r="C98">
         <v>3</v>
       </c>
+      <c r="D98" t="s">
+        <v>181</v>
+      </c>
       <c r="E98" t="s">
         <v>155</v>
       </c>
@@ -2615,6 +2680,9 @@
       <c r="C99">
         <v>3</v>
       </c>
+      <c r="D99" t="s">
+        <v>149</v>
+      </c>
       <c r="E99" t="s">
         <v>156</v>
       </c>
@@ -2628,6 +2696,9 @@
       </c>
       <c r="C100">
         <v>3</v>
+      </c>
+      <c r="D100" s="7" t="s">
+        <v>153</v>
       </c>
       <c r="E100" t="s">
         <v>154</v>

</xml_diff>